<commit_message>
Completed excel to python notebook with all 4 projects python code and markdown explanations
</commit_message>
<xml_diff>
--- a/Excel_HandsON.xlsx
+++ b/Excel_HandsON.xlsx
@@ -5,12 +5,12 @@
   <workbookPr hidePivotFieldList="1"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/ayaanjauhar/Downloads/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/ayaanjauhar/excel_python_project/"/>
     </mc:Choice>
   </mc:AlternateContent>
   <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0FE00282-2EB2-FF46-9703-819FDF180ACE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="580" windowWidth="28800" windowHeight="18060" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="580" windowWidth="28800" windowHeight="16560" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Read me" sheetId="1" r:id="rId1"/>
@@ -22,7 +22,7 @@
   </sheets>
   <calcPr calcId="191029"/>
   <pivotCaches>
-    <pivotCache cacheId="5" r:id="rId7"/>
+    <pivotCache cacheId="0" r:id="rId7"/>
   </pivotCaches>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
@@ -350,7 +350,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="18">
+  <cellXfs count="17">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -375,7 +375,6 @@
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" pivotButton="1"/>
     <xf numFmtId="10" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="8" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" readingOrder="1"/>
     </xf>
@@ -462,7 +461,7 @@
               <a:cs typeface="+mn-cs"/>
             </a:defRPr>
           </a:pPr>
-          <a:endParaRPr lang="en-US"/>
+          <a:endParaRPr lang="en-GB"/>
         </a:p>
       </c:txPr>
     </c:title>
@@ -615,7 +614,7 @@
                   <a:cs typeface="+mn-cs"/>
                 </a:defRPr>
               </a:pPr>
-              <a:endParaRPr lang="en-US"/>
+              <a:endParaRPr lang="en-GB"/>
             </a:p>
           </c:txPr>
         </c:title>
@@ -900,7 +899,7 @@
               <a:cs typeface="+mn-cs"/>
             </a:defRPr>
           </a:pPr>
-          <a:endParaRPr lang="en-US"/>
+          <a:endParaRPr lang="en-GB"/>
         </a:p>
       </c:txPr>
     </c:title>
@@ -926,6 +925,11 @@
               </a:ln>
               <a:effectLst/>
             </c:spPr>
+            <c:extLst>
+              <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                <c16:uniqueId val="{00000001-2785-C04D-9655-2D3B5A27F6D1}"/>
+              </c:ext>
+            </c:extLst>
           </c:dPt>
           <c:dPt>
             <c:idx val="1"/>
@@ -941,6 +945,11 @@
               </a:ln>
               <a:effectLst/>
             </c:spPr>
+            <c:extLst>
+              <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                <c16:uniqueId val="{00000003-2785-C04D-9655-2D3B5A27F6D1}"/>
+              </c:ext>
+            </c:extLst>
           </c:dPt>
           <c:dPt>
             <c:idx val="2"/>
@@ -956,6 +965,11 @@
               </a:ln>
               <a:effectLst/>
             </c:spPr>
+            <c:extLst>
+              <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                <c16:uniqueId val="{00000005-2785-C04D-9655-2D3B5A27F6D1}"/>
+              </c:ext>
+            </c:extLst>
           </c:dPt>
           <c:dPt>
             <c:idx val="3"/>
@@ -971,6 +985,11 @@
               </a:ln>
               <a:effectLst/>
             </c:spPr>
+            <c:extLst>
+              <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                <c16:uniqueId val="{00000007-2785-C04D-9655-2D3B5A27F6D1}"/>
+              </c:ext>
+            </c:extLst>
           </c:dPt>
           <c:dPt>
             <c:idx val="4"/>
@@ -986,6 +1005,11 @@
               </a:ln>
               <a:effectLst/>
             </c:spPr>
+            <c:extLst>
+              <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                <c16:uniqueId val="{00000009-2785-C04D-9655-2D3B5A27F6D1}"/>
+              </c:ext>
+            </c:extLst>
           </c:dPt>
           <c:dLbls>
             <c:spPr>
@@ -1437,7 +1461,7 @@
                   <a:cs typeface="+mn-cs"/>
                 </a:defRPr>
               </a:pPr>
-              <a:endParaRPr lang="en-US"/>
+              <a:endParaRPr lang="en-GB"/>
             </a:p>
           </c:txPr>
         </c:title>
@@ -2066,6 +2090,230 @@
       </c:pivotFmt>
       <c:pivotFmt>
         <c:idx val="7"/>
+        <c:spPr>
+          <a:solidFill>
+            <a:schemeClr val="accent1"/>
+          </a:solidFill>
+          <a:ln>
+            <a:noFill/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:marker>
+          <c:symbol val="none"/>
+        </c:marker>
+        <c:dLbl>
+          <c:idx val="0"/>
+          <c:spPr>
+            <a:noFill/>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:txPr>
+            <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr" anchorCtr="1">
+              <a:spAutoFit/>
+            </a:bodyPr>
+            <a:lstStyle/>
+            <a:p>
+              <a:pPr>
+                <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                  <a:solidFill>
+                    <a:schemeClr val="tx1">
+                      <a:lumMod val="75000"/>
+                      <a:lumOff val="25000"/>
+                    </a:schemeClr>
+                  </a:solidFill>
+                  <a:latin typeface="+mn-lt"/>
+                  <a:ea typeface="+mn-ea"/>
+                  <a:cs typeface="+mn-cs"/>
+                </a:defRPr>
+              </a:pPr>
+              <a:endParaRPr lang="en-US"/>
+            </a:p>
+          </c:txPr>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="0"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+          <c:showBubbleSize val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}"/>
+          </c:extLst>
+        </c:dLbl>
+      </c:pivotFmt>
+      <c:pivotFmt>
+        <c:idx val="8"/>
+        <c:spPr>
+          <a:solidFill>
+            <a:schemeClr val="accent1"/>
+          </a:solidFill>
+          <a:ln>
+            <a:noFill/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:marker>
+          <c:symbol val="none"/>
+        </c:marker>
+        <c:dLbl>
+          <c:idx val="0"/>
+          <c:spPr>
+            <a:noFill/>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:txPr>
+            <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr" anchorCtr="1">
+              <a:spAutoFit/>
+            </a:bodyPr>
+            <a:lstStyle/>
+            <a:p>
+              <a:pPr>
+                <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                  <a:solidFill>
+                    <a:schemeClr val="tx1">
+                      <a:lumMod val="75000"/>
+                      <a:lumOff val="25000"/>
+                    </a:schemeClr>
+                  </a:solidFill>
+                  <a:latin typeface="+mn-lt"/>
+                  <a:ea typeface="+mn-ea"/>
+                  <a:cs typeface="+mn-cs"/>
+                </a:defRPr>
+              </a:pPr>
+              <a:endParaRPr lang="en-US"/>
+            </a:p>
+          </c:txPr>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="0"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+          <c:showBubbleSize val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}"/>
+          </c:extLst>
+        </c:dLbl>
+      </c:pivotFmt>
+      <c:pivotFmt>
+        <c:idx val="9"/>
+        <c:spPr>
+          <a:solidFill>
+            <a:schemeClr val="accent1"/>
+          </a:solidFill>
+          <a:ln>
+            <a:noFill/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:marker>
+          <c:symbol val="none"/>
+        </c:marker>
+        <c:dLbl>
+          <c:idx val="0"/>
+          <c:spPr>
+            <a:noFill/>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:txPr>
+            <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr" anchorCtr="1">
+              <a:spAutoFit/>
+            </a:bodyPr>
+            <a:lstStyle/>
+            <a:p>
+              <a:pPr>
+                <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                  <a:solidFill>
+                    <a:schemeClr val="tx1">
+                      <a:lumMod val="75000"/>
+                      <a:lumOff val="25000"/>
+                    </a:schemeClr>
+                  </a:solidFill>
+                  <a:latin typeface="+mn-lt"/>
+                  <a:ea typeface="+mn-ea"/>
+                  <a:cs typeface="+mn-cs"/>
+                </a:defRPr>
+              </a:pPr>
+              <a:endParaRPr lang="en-US"/>
+            </a:p>
+          </c:txPr>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="0"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+          <c:showBubbleSize val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}"/>
+          </c:extLst>
+        </c:dLbl>
+      </c:pivotFmt>
+      <c:pivotFmt>
+        <c:idx val="10"/>
+        <c:spPr>
+          <a:solidFill>
+            <a:schemeClr val="accent1"/>
+          </a:solidFill>
+          <a:ln>
+            <a:noFill/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:marker>
+          <c:symbol val="none"/>
+        </c:marker>
+        <c:dLbl>
+          <c:idx val="0"/>
+          <c:spPr>
+            <a:noFill/>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:txPr>
+            <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr" anchorCtr="1">
+              <a:spAutoFit/>
+            </a:bodyPr>
+            <a:lstStyle/>
+            <a:p>
+              <a:pPr>
+                <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                  <a:solidFill>
+                    <a:schemeClr val="tx1">
+                      <a:lumMod val="75000"/>
+                      <a:lumOff val="25000"/>
+                    </a:schemeClr>
+                  </a:solidFill>
+                  <a:latin typeface="+mn-lt"/>
+                  <a:ea typeface="+mn-ea"/>
+                  <a:cs typeface="+mn-cs"/>
+                </a:defRPr>
+              </a:pPr>
+              <a:endParaRPr lang="en-US"/>
+            </a:p>
+          </c:txPr>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="0"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+          <c:showBubbleSize val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}"/>
+          </c:extLst>
+        </c:dLbl>
+      </c:pivotFmt>
+      <c:pivotFmt>
+        <c:idx val="11"/>
         <c:spPr>
           <a:solidFill>
             <a:schemeClr val="accent1"/>
@@ -4060,7 +4308,7 @@
               <a:cs typeface="+mn-cs"/>
             </a:defRPr>
           </a:pPr>
-          <a:endParaRPr lang="en-US"/>
+          <a:endParaRPr lang="en-GB"/>
         </a:p>
       </c:txPr>
     </c:title>
@@ -4352,7 +4600,7 @@
                   <a:cs typeface="+mn-cs"/>
                 </a:defRPr>
               </a:pPr>
-              <a:endParaRPr lang="en-US"/>
+              <a:endParaRPr lang="en-GB"/>
             </a:p>
           </c:txPr>
         </c:title>
@@ -4470,7 +4718,7 @@
                   <a:cs typeface="+mn-cs"/>
                 </a:defRPr>
               </a:pPr>
-              <a:endParaRPr lang="en-US"/>
+              <a:endParaRPr lang="en-GB"/>
             </a:p>
           </c:txPr>
         </c:title>
@@ -9266,7 +9514,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable1.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{5B0582A1-A1D4-4246-A1D5-E5277966D7D5}" name="PivotTable3" cacheId="5" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="4">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{5B0582A1-A1D4-4246-A1D5-E5277966D7D5}" name="PivotTable3" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="4">
   <location ref="A39:F43" firstHeaderRow="1" firstDataRow="2" firstDataCol="1"/>
   <pivotFields count="4">
     <pivotField showAll="0"/>
@@ -9551,7 +9799,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable2.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{5FCB5F3E-1A90-FD40-BB4B-15E94B2FEDDC}" name="PivotTable2" cacheId="5" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="11">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{5FCB5F3E-1A90-FD40-BB4B-15E94B2FEDDC}" name="PivotTable2" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="11">
   <location ref="A22:F26" firstHeaderRow="1" firstDataRow="2" firstDataCol="1"/>
   <pivotFields count="4">
     <pivotField showAll="0"/>
@@ -10016,7 +10264,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable3.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{0FC15581-13F8-BB4B-9796-7C1868BC348C}" name="PivotTable1" cacheId="5" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="2">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{0FC15581-13F8-BB4B-9796-7C1868BC348C}" name="PivotTable1" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="2">
   <location ref="A3:F7" firstHeaderRow="1" firstDataRow="2" firstDataCol="1"/>
   <pivotFields count="4">
     <pivotField showAll="0"/>
@@ -10154,7 +10402,7 @@
   <dataFields count="1">
     <dataField name="Count of Brand" fld="1" subtotal="count" baseField="0" baseItem="0"/>
   </dataFields>
-  <chartFormats count="8">
+  <chartFormats count="12">
     <chartFormat chart="0" format="4" series="1">
       <pivotArea type="data" outline="0" fieldPosition="0">
         <references count="1">
@@ -10228,6 +10476,54 @@
       </pivotArea>
     </chartFormat>
     <chartFormat chart="1" format="3" series="1">
+      <pivotArea type="data" outline="0" fieldPosition="0">
+        <references count="2">
+          <reference field="4294967294" count="1" selected="0">
+            <x v="0"/>
+          </reference>
+          <reference field="1" count="1" selected="0">
+            <x v="3"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </chartFormat>
+    <chartFormat chart="0" format="8" series="1">
+      <pivotArea type="data" outline="0" fieldPosition="0">
+        <references count="2">
+          <reference field="4294967294" count="1" selected="0">
+            <x v="0"/>
+          </reference>
+          <reference field="1" count="1" selected="0">
+            <x v="0"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </chartFormat>
+    <chartFormat chart="0" format="9" series="1">
+      <pivotArea type="data" outline="0" fieldPosition="0">
+        <references count="2">
+          <reference field="4294967294" count="1" selected="0">
+            <x v="0"/>
+          </reference>
+          <reference field="1" count="1" selected="0">
+            <x v="1"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </chartFormat>
+    <chartFormat chart="0" format="10" series="1">
+      <pivotArea type="data" outline="0" fieldPosition="0">
+        <references count="2">
+          <reference field="4294967294" count="1" selected="0">
+            <x v="0"/>
+          </reference>
+          <reference field="1" count="1" selected="0">
+            <x v="2"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </chartFormat>
+    <chartFormat chart="0" format="11" series="1">
       <pivotArea type="data" outline="0" fieldPosition="0">
         <references count="2">
           <reference field="4294967294" count="1" selected="0">
@@ -10658,7 +10954,7 @@
         <v>9</v>
       </c>
       <c r="E3">
-        <f t="shared" ref="E3:E7" si="0">COUNTIF($B$2:$B$41, D3)</f>
+        <f t="shared" ref="E3:E6" si="0">COUNTIF($B$2:$B$41, D3)</f>
         <v>9</v>
       </c>
       <c r="F3">
@@ -11866,19 +12162,19 @@
       <c r="A5" s="10" t="s">
         <v>65</v>
       </c>
-      <c r="B5" s="16">
+      <c r="B5">
         <v>16</v>
       </c>
-      <c r="C5" s="16">
+      <c r="C5">
         <v>8</v>
       </c>
-      <c r="D5" s="16">
+      <c r="D5">
         <v>6</v>
       </c>
-      <c r="E5" s="16">
+      <c r="E5">
         <v>6</v>
       </c>
-      <c r="F5" s="16">
+      <c r="F5">
         <v>36</v>
       </c>
     </row>
@@ -11886,19 +12182,19 @@
       <c r="A6" s="10" t="s">
         <v>64</v>
       </c>
-      <c r="B6" s="16">
+      <c r="B6">
         <v>2</v>
       </c>
-      <c r="C6" s="16">
+      <c r="C6">
         <v>12</v>
       </c>
-      <c r="D6" s="16">
+      <c r="D6">
         <v>14</v>
       </c>
-      <c r="E6" s="16">
+      <c r="E6">
         <v>16</v>
       </c>
-      <c r="F6" s="16">
+      <c r="F6">
         <v>44</v>
       </c>
     </row>
@@ -11906,19 +12202,19 @@
       <c r="A7" s="10" t="s">
         <v>62</v>
       </c>
-      <c r="B7" s="16">
+      <c r="B7">
         <v>18</v>
       </c>
-      <c r="C7" s="16">
+      <c r="C7">
         <v>20</v>
       </c>
-      <c r="D7" s="16">
+      <c r="D7">
         <v>20</v>
       </c>
-      <c r="E7" s="16">
+      <c r="E7">
         <v>22</v>
       </c>
-      <c r="F7" s="16">
+      <c r="F7">
         <v>80</v>
       </c>
     </row>
@@ -13492,7 +13788,7 @@
       <c r="D13" s="13" t="s">
         <v>67</v>
       </c>
-      <c r="E13" s="17">
+      <c r="E13" s="16">
         <f xml:space="preserve"> 5.2454*7 + 23.447</f>
         <v>60.1648</v>
       </c>

</xml_diff>